<commit_message>
feat: Customize Genset numerical readings form and logs with the 8 user questions
</commit_message>
<xml_diff>
--- a/genset_readings_log.xlsx
+++ b/genset_readings_log.xlsx
@@ -1250,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1268,9 +1268,8 @@
       <c r="E1" s="23" t="n"/>
       <c r="F1" s="23" t="n"/>
       <c r="G1" s="23" t="n"/>
-      <c r="H1" s="23" t="n"/>
-      <c r="I1" s="24" t="n"/>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="H1" s="24" t="n"/>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DOC NO: R/MAI/GR
 MONTH/YEAR: </t>
@@ -1290,8 +1289,7 @@
       <c r="F2" s="25" t="n"/>
       <c r="G2" s="25" t="n"/>
       <c r="H2" s="25" t="n"/>
-      <c r="I2" s="25" t="n"/>
-      <c r="J2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1301,47 +1299,42 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>RUN HOURS</t>
+          <t>BATTERY VOLTAGE</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>COOLANT TEMP</t>
+          <t>DIESEL FILLING (LTR)</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>LUBE OIL PRESS</t>
+          <t>RUNNING HOURS</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>FUEL LEVEL</t>
+          <t>VOLTAGE</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>BATTERY VOLT</t>
+          <t>KW/H</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>VOLT R</t>
+          <t>DIESEL LEVEL</t>
         </is>
       </c>
       <c r="H3" s="10" t="inlineStr">
         <is>
-          <t>VOLT Y</t>
+          <t>RADIATOR WATER</t>
         </is>
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>VOLT B</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>FREQ</t>
+          <t>CARETAKER SIGN</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1350,6 @@
       <c r="G4" s="13" t="n"/>
       <c r="H4" s="13" t="n"/>
       <c r="I4" s="13" t="n"/>
-      <c r="J4" s="13" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="12" t="n">
@@ -1371,7 +1363,6 @@
       <c r="G5" s="13" t="n"/>
       <c r="H5" s="13" t="n"/>
       <c r="I5" s="13" t="n"/>
-      <c r="J5" s="13" t="n"/>
     </row>
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="12" t="n">
@@ -1385,7 +1376,6 @@
       <c r="G6" s="13" t="n"/>
       <c r="H6" s="13" t="n"/>
       <c r="I6" s="13" t="n"/>
-      <c r="J6" s="13" t="n"/>
     </row>
     <row r="7" ht="33" customHeight="1">
       <c r="A7" s="12" t="n">
@@ -1399,7 +1389,6 @@
       <c r="G7" s="13" t="n"/>
       <c r="H7" s="13" t="n"/>
       <c r="I7" s="13" t="n"/>
-      <c r="J7" s="13" t="n"/>
     </row>
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -1413,7 +1402,6 @@
       <c r="G8" s="13" t="n"/>
       <c r="H8" s="13" t="n"/>
       <c r="I8" s="13" t="n"/>
-      <c r="J8" s="13" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="12" t="n">
@@ -1427,7 +1415,6 @@
       <c r="G9" s="13" t="n"/>
       <c r="H9" s="13" t="n"/>
       <c r="I9" s="13" t="n"/>
-      <c r="J9" s="13" t="n"/>
     </row>
     <row r="10" ht="33" customHeight="1">
       <c r="A10" s="15" t="n">
@@ -1441,7 +1428,6 @@
       <c r="G10" s="16" t="n"/>
       <c r="H10" s="16" t="n"/>
       <c r="I10" s="16" t="n"/>
-      <c r="J10" s="16" t="n"/>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="12" t="n">
@@ -1455,7 +1441,6 @@
       <c r="G11" s="13" t="n"/>
       <c r="H11" s="13" t="n"/>
       <c r="I11" s="13" t="n"/>
-      <c r="J11" s="13" t="n"/>
     </row>
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="12" t="n">
@@ -1469,7 +1454,6 @@
       <c r="G12" s="13" t="n"/>
       <c r="H12" s="13" t="n"/>
       <c r="I12" s="13" t="n"/>
-      <c r="J12" s="13" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="12" t="n">
@@ -1483,7 +1467,6 @@
       <c r="G13" s="13" t="n"/>
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="13" t="n"/>
-      <c r="J13" s="13" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="12" t="n">
@@ -1497,7 +1480,6 @@
       <c r="G14" s="13" t="n"/>
       <c r="H14" s="13" t="n"/>
       <c r="I14" s="13" t="n"/>
-      <c r="J14" s="13" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="12" t="n">
@@ -1511,7 +1493,6 @@
       <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="13" t="n"/>
-      <c r="J15" s="13" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="12" t="n">
@@ -1525,7 +1506,6 @@
       <c r="G16" s="13" t="n"/>
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="13" t="n"/>
-      <c r="J16" s="13" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="15" t="n">
@@ -1539,7 +1519,6 @@
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="16" t="n"/>
       <c r="I17" s="16" t="n"/>
-      <c r="J17" s="16" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1">
       <c r="A18" s="12" t="n">
@@ -1553,7 +1532,6 @@
       <c r="G18" s="13" t="n"/>
       <c r="H18" s="13" t="n"/>
       <c r="I18" s="13" t="n"/>
-      <c r="J18" s="13" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1">
       <c r="A19" s="6" t="n"/>
@@ -1568,8 +1546,7 @@
       <c r="F19" s="25" t="n"/>
       <c r="G19" s="25" t="n"/>
       <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
-      <c r="J19" s="26" t="n"/>
+      <c r="I19" s="26" t="n"/>
     </row>
     <row r="20" ht="59.25" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1579,47 +1556,42 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>RUN HOURS</t>
+          <t>BATTERY VOLTAGE</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>COOLANT TEMP</t>
+          <t>DIESEL FILLING (LTR)</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>LUBE OIL PRESS</t>
+          <t>RUNNING HOURS</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>FUEL LEVEL</t>
+          <t>VOLTAGE</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>BATTERY VOLT</t>
+          <t>KW/H</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>VOLT R</t>
+          <t>DIESEL LEVEL</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>VOLT Y</t>
+          <t>RADIATOR WATER</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>VOLT B</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>FREQ</t>
+          <t>CARETAKER SIGN</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1607,6 @@
       <c r="G21" s="13" t="n"/>
       <c r="H21" s="13" t="n"/>
       <c r="I21" s="13" t="n"/>
-      <c r="J21" s="13" t="n"/>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="12" t="n">
@@ -1649,7 +1620,6 @@
       <c r="G22" s="13" t="n"/>
       <c r="H22" s="13" t="n"/>
       <c r="I22" s="13" t="n"/>
-      <c r="J22" s="13" t="n"/>
     </row>
     <row r="23" ht="33" customHeight="1">
       <c r="A23" s="12" t="n">
@@ -1663,7 +1633,6 @@
       <c r="G23" s="13" t="n"/>
       <c r="H23" s="13" t="n"/>
       <c r="I23" s="13" t="n"/>
-      <c r="J23" s="13" t="n"/>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="12" t="n">
@@ -1677,7 +1646,6 @@
       <c r="G24" s="13" t="n"/>
       <c r="H24" s="13" t="n"/>
       <c r="I24" s="13" t="n"/>
-      <c r="J24" s="13" t="n"/>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="12" t="n">
@@ -1691,7 +1659,6 @@
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n"/>
       <c r="I25" s="13" t="n"/>
-      <c r="J25" s="13" t="n"/>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="A26" s="15" t="n">
@@ -1705,7 +1672,6 @@
       <c r="G26" s="16" t="n"/>
       <c r="H26" s="16" t="n"/>
       <c r="I26" s="16" t="n"/>
-      <c r="J26" s="16" t="n"/>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="12" t="n">
@@ -1719,7 +1685,6 @@
       <c r="G27" s="13" t="n"/>
       <c r="H27" s="13" t="n"/>
       <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
     </row>
     <row r="28" ht="33" customHeight="1">
       <c r="A28" s="12" t="n">
@@ -1733,7 +1698,6 @@
       <c r="G28" s="13" t="n"/>
       <c r="H28" s="13" t="n"/>
       <c r="I28" s="13" t="n"/>
-      <c r="J28" s="13" t="n"/>
     </row>
     <row r="29" ht="33" customHeight="1">
       <c r="A29" s="12" t="n">
@@ -1747,7 +1711,6 @@
       <c r="G29" s="13" t="n"/>
       <c r="H29" s="13" t="n"/>
       <c r="I29" s="13" t="n"/>
-      <c r="J29" s="13" t="n"/>
     </row>
     <row r="30" ht="33" customHeight="1">
       <c r="A30" s="12" t="n">
@@ -1761,7 +1724,6 @@
       <c r="G30" s="13" t="n"/>
       <c r="H30" s="13" t="n"/>
       <c r="I30" s="13" t="n"/>
-      <c r="J30" s="13" t="n"/>
     </row>
     <row r="31" ht="33" customHeight="1">
       <c r="A31" s="12" t="n">
@@ -1775,7 +1737,6 @@
       <c r="G31" s="13" t="n"/>
       <c r="H31" s="13" t="n"/>
       <c r="I31" s="13" t="n"/>
-      <c r="J31" s="13" t="n"/>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="A32" s="12" t="n">
@@ -1789,7 +1750,6 @@
       <c r="G32" s="13" t="n"/>
       <c r="H32" s="13" t="n"/>
       <c r="I32" s="13" t="n"/>
-      <c r="J32" s="13" t="n"/>
     </row>
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="15" t="n">
@@ -1803,7 +1763,6 @@
       <c r="G33" s="16" t="n"/>
       <c r="H33" s="16" t="n"/>
       <c r="I33" s="16" t="n"/>
-      <c r="J33" s="16" t="n"/>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="12" t="n">
@@ -1817,7 +1776,6 @@
       <c r="G34" s="13" t="n"/>
       <c r="H34" s="13" t="n"/>
       <c r="I34" s="13" t="n"/>
-      <c r="J34" s="13" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" thickBot="1">
       <c r="A35" s="12" t="n">
@@ -1831,7 +1789,6 @@
       <c r="G35" s="13" t="n"/>
       <c r="H35" s="13" t="n"/>
       <c r="I35" s="13" t="n"/>
-      <c r="J35" s="13" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1"/>
     <row r="37" ht="48.75" customHeight="1"/>
@@ -1849,10 +1806,10 @@
     <row r="55" ht="45" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="J1"/>
-    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>